<commit_message>
chore(data): sync map records with updated bin survey
Update the source Excel file and regenerate the embedded `records` dataset in `index.html` to reflect the latest public trash-bin coordinates and metadata. This keeps the map data aligned with the most recent field updates.chore(data): sync map records with updated bin survey

Update the source Excel file and regenerate the embedded `records` dataset in `index.html` to reflect the latest public trash-bin coordinates and metadata. This keeps the map data aligned with the most recent field updates.
</commit_message>
<xml_diff>
--- a/Bssy_coordonnees_completes_poubelles publiques v0.xlsx
+++ b/Bssy_coordonnees_completes_poubelles publiques v0.xlsx
@@ -544,9 +544,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F50"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" ns3:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.1796875" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -556,7 +556,7 @@
     <col min="6" max="6" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="18.5" ns3:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -576,7 +576,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ns3:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -593,7 +593,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ns3:dyDescent="0.35">
       <c r="A3">
         <f>A2+1</f>
         <v>2</v>
@@ -611,7 +611,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" ns3:dyDescent="0.35">
       <c r="A4">
         <f t="shared" ref="A4:A45" si="0">A3+1</f>
         <v>3</v>
@@ -629,7 +629,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" ns3:dyDescent="0.35">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -647,7 +647,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" ns3:dyDescent="0.35">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -665,7 +665,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" ns3:dyDescent="0.35">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -683,7 +683,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" ns3:dyDescent="0.35">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -701,7 +701,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" ns3:dyDescent="0.35">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -719,7 +719,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" ns3:dyDescent="0.35">
       <c r="A10" s="1">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -737,7 +737,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" ns3:dyDescent="0.35">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -755,7 +755,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" ns3:dyDescent="0.35">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -773,7 +773,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" ns3:dyDescent="0.35">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -791,7 +791,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" ns3:dyDescent="0.35">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -809,7 +809,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" ns3:dyDescent="0.35">
       <c r="A15">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -827,7 +827,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" ns3:dyDescent="0.35">
       <c r="A16">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -845,7 +845,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" ns3:dyDescent="0.35">
       <c r="A17">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -863,7 +863,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" ns3:dyDescent="0.35">
       <c r="A18">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -881,7 +881,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" ns3:dyDescent="0.35">
       <c r="A19">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -899,7 +899,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" ns3:dyDescent="0.35">
       <c r="A20">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -917,7 +917,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" ns3:dyDescent="0.35">
       <c r="A21">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -935,7 +935,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" ns3:dyDescent="0.35">
       <c r="A22">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -953,7 +953,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" ns3:dyDescent="0.35">
       <c r="A23">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -971,7 +971,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" ns3:dyDescent="0.35">
       <c r="A24">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -989,7 +989,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" ns3:dyDescent="0.35">
       <c r="A25">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -1007,7 +1007,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" ns3:dyDescent="0.35">
       <c r="A26">
         <f t="shared" si="0"/>
         <v>25</v>
@@ -1025,16 +1025,16 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" ns3:dyDescent="0.35">
       <c r="A27">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="B27">
-        <v>48.549300000000002</v>
+        <v>48.548728</v>
       </c>
       <c r="C27">
-        <v>2.2093666999999999</v>
+        <v>2.208855</v>
       </c>
       <c r="D27">
         <v>140</v>
@@ -1043,7 +1043,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" ns3:dyDescent="0.35">
       <c r="A28" s="1">
         <f t="shared" si="0"/>
         <v>27</v>
@@ -1061,7 +1061,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" ns3:dyDescent="0.35">
       <c r="A29">
         <f t="shared" si="0"/>
         <v>28</v>
@@ -1079,7 +1079,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" ns3:dyDescent="0.35">
       <c r="A30">
         <f t="shared" si="0"/>
         <v>29</v>
@@ -1097,7 +1097,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" ns3:dyDescent="0.35">
       <c r="A31">
         <f t="shared" si="0"/>
         <v>30</v>
@@ -1115,16 +1115,16 @@
         <v>24</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" ns3:dyDescent="0.35">
       <c r="A32">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="B32">
-        <v>48.548558300000003</v>
+        <v>48.548728</v>
       </c>
       <c r="C32">
-        <v>2.2087967000000002</v>
+        <v>2.208855</v>
       </c>
       <c r="D32">
         <v>139</v>
@@ -1133,7 +1133,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" ns3:dyDescent="0.35">
       <c r="A33">
         <f t="shared" si="0"/>
         <v>32</v>
@@ -1151,7 +1151,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" ns3:dyDescent="0.35">
       <c r="A34">
         <f t="shared" si="0"/>
         <v>33</v>
@@ -1169,7 +1169,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" ns3:dyDescent="0.35">
       <c r="A35" s="1">
         <f t="shared" si="0"/>
         <v>34</v>
@@ -1187,7 +1187,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" ns3:dyDescent="0.35">
       <c r="A36">
         <f t="shared" si="0"/>
         <v>35</v>
@@ -1205,7 +1205,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" ns3:dyDescent="0.35">
       <c r="A37">
         <f t="shared" si="0"/>
         <v>36</v>
@@ -1223,7 +1223,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" ns3:dyDescent="0.35">
       <c r="A38">
         <f t="shared" si="0"/>
         <v>37</v>
@@ -1241,7 +1241,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" ns3:dyDescent="0.35">
       <c r="A39">
         <f t="shared" si="0"/>
         <v>38</v>
@@ -1259,7 +1259,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" ns3:dyDescent="0.35">
       <c r="A40">
         <f t="shared" si="0"/>
         <v>39</v>
@@ -1277,7 +1277,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" ns3:dyDescent="0.35">
       <c r="A41">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -1295,7 +1295,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" ns3:dyDescent="0.35">
       <c r="A42">
         <f t="shared" si="0"/>
         <v>41</v>
@@ -1313,7 +1313,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" ns3:dyDescent="0.35">
       <c r="A43">
         <f t="shared" si="0"/>
         <v>42</v>
@@ -1331,7 +1331,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" ns3:dyDescent="0.35">
       <c r="A44">
         <f t="shared" si="0"/>
         <v>43</v>
@@ -1349,7 +1349,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" ns3:dyDescent="0.35">
       <c r="A45">
         <f t="shared" si="0"/>
         <v>44</v>
@@ -1367,7 +1367,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" ns3:dyDescent="0.35">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1384,7 +1384,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" ns3:dyDescent="0.35">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1401,7 +1401,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" ns3:dyDescent="0.35">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1418,7 +1418,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" ns3:dyDescent="0.35">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1435,7 +1435,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" ns3:dyDescent="0.35">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1454,6 +1454,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" ns4:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(data): refresh public bin coordinates and map records
Update the source Excel file and regenerate the embedded `records` data in `index.html` to reflect the latest bin locations and associated photo metadata. This keeps the published map aligned with the most recent field data.chore(data): refresh public bin coordinates and map records

Update the source Excel file and regenerate the embedded `records` data in `index.html` to reflect the latest bin locations and associated photo metadata. This keeps the published map aligned with the most recent field data.
</commit_message>
<xml_diff>
--- a/Bssy_coordonnees_completes_poubelles publiques v0.xlsx
+++ b/Bssy_coordonnees_completes_poubelles publiques v0.xlsx
@@ -1031,10 +1031,10 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>48.548728</v>
+        <v>48.549329</v>
       </c>
       <c r="C27">
-        <v>2.208855</v>
+        <v>2.20996</v>
       </c>
       <c r="D27">
         <v>140</v>
@@ -1193,10 +1193,10 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>48.549548799999997</v>
+        <v>48.549375</v>
       </c>
       <c r="C36">
-        <v>2.2108235999999999</v>
+        <v>2.210652</v>
       </c>
       <c r="D36">
         <v>139</v>

</xml_diff>